<commit_message>
feat(import-cli): multi-supplier support via an optional "Pemasok Produk" sheet
The new optional sheet carries the *additional* suppliers per item
(`Produk.nama_pemasok` still means "preferred"), making this the first import
path able to populate `supplierItemCode`, `ItemSupplier.cost` and
`leadTimeDays`. Old filled templates import unchanged.

Adds a Global-DB Pro plan check to the direct importer: `--direct` bypasses
`syncItemSuppliers` and with it the second-supplier guard, so the gate has to
be re-asserted locally.

Operator-run tool only — not deployed, no migration, no APK. Ship note:
re-send `TEMPLATE_KOSONG.xlsx` + `PANDUAN_PENGISIAN` to any tenant mid-
onboarding so they pick up the new tab.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/import-cli/templates/CONTOH_TERISI.xlsx
+++ b/tools/import-cli/templates/CONTOH_TERISI.xlsx
@@ -8,14 +8,15 @@
     <sheet sheetId="2" name="Pemasok" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Produk" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="Varian Produk" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Pelanggan" state="visible" r:id="rId8"/>
+    <sheet sheetId="5" name="Pemasok Produk" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Pelanggan" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="75">
   <si>
     <t>nama_kategori</t>
   </si>
@@ -98,6 +99,30 @@
     <t>Ya</t>
   </si>
   <si>
+    <t>CV Sumber Rejeki</t>
+  </si>
+  <si>
+    <t>Bandung</t>
+  </si>
+  <si>
+    <t>Jawa Barat</t>
+  </si>
+  <si>
+    <t>Budi</t>
+  </si>
+  <si>
+    <t>+628987654321</t>
+  </si>
+  <si>
+    <t>budi@sumberrejeki.co.id</t>
+  </si>
+  <si>
+    <t>Tidak</t>
+  </si>
+  <si>
+    <t>Pemasok cadangan</t>
+  </si>
+  <si>
     <t>nama_produk</t>
   </si>
   <si>
@@ -146,9 +171,6 @@
     <t>Segitiga Biru</t>
   </si>
   <si>
-    <t>Tidak</t>
-  </si>
-  <si>
     <t>Gula Pasir 1kg</t>
   </si>
   <si>
@@ -189,6 +211,18 @@
   </si>
   <si>
     <t>nilai_atribut_2</t>
+  </si>
+  <si>
+    <t>kode_produk_pemasok</t>
+  </si>
+  <si>
+    <t>lead_time_hari</t>
+  </si>
+  <si>
+    <t>SR-TERIGU-1</t>
+  </si>
+  <si>
+    <t>SR-GULA-1</t>
   </si>
   <si>
     <t>nama_depan</t>
@@ -739,7 +773,35 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="8:8" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
     <row r="4" spans="8:8" x14ac:dyDescent="0.25"/>
     <row r="5" spans="8:8" x14ac:dyDescent="0.25"/>
     <row r="6" spans="8:8" x14ac:dyDescent="0.25"/>
@@ -972,10 +1034,10 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -984,42 +1046,42 @@
         <v>10</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>17</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>3</v>
@@ -1037,19 +1099,19 @@
         <v>50</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>26</v>
@@ -1060,10 +1122,10 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>3</v>
@@ -1081,19 +1143,19 @@
         <v>40</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>5</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>26</v>
@@ -1104,10 +1166,10 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>6</v>
@@ -1125,19 +1187,19 @@
         <v>100</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>26</v>
@@ -1388,37 +1450,37 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25"/>
@@ -1649,6 +1711,286 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E201"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="26" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="5" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2" s="3">
+        <v>12500</v>
+      </c>
+      <c r="E2" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" s="3">
+        <v>13200</v>
+      </c>
+      <c r="E3" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="172" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="175" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="191" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Tidak valid" error="Pilih nilai dari daftar." sqref="A10:A201">
+      <formula1>Produk!$B$2:$B$201</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Tidak valid" error="Pilih nilai dari daftar." sqref="A2:A201">
+      <formula1>Produk!$B$2:$B$201</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Tidak valid" error="Pilih nilai dari daftar." sqref="B10:B201">
+      <formula1>Pemasok!$A$2:$A$201</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Tidak valid" error="Pilih nilai dari daftar." sqref="B2:B201">
+      <formula1>Pemasok!$A$2:$A$201</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -1660,10 +2002,10 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>15</v>
@@ -1677,16 +2019,16 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>20</v>

</xml_diff>